<commit_message>
Ajouter le graphique d'evolution des sessions au rapport hebdo (06/07-12/07)
Execution hors cycle du 18/07/2026 : aucune nouvelle semaine calendaire
complete n'ayant pu s'ecouler depuis le rapport du 17/07/2026, ce rafraichissement
porte sur la meme semaine et ajoute le graphique natif Excel (5 semaines
disponibles depuis la creation de la propriete GA4 le 08/06/2026, cf. §10.1).
Toutes les donnees GA4/Search Console/Semrush ont ete revérifiées en direct
et sont inchangees (hors deux compteurs mineurs Semrush pour sealsystems.fr).
recalc.py a expire apres 150s (tentative unique, non renouvelee) : formules
standard, calcul normal a l'ouverture Excel.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017AWWewxDRVc1g3LLVvTpNS
</commit_message>
<xml_diff>
--- a/reports/rapport-2026-07-06_2026-07-12.xlsx
+++ b/reports/rapport-2026-07-06_2026-07-12.xlsx
@@ -19,12 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="+0.0%;-0.0%;0.0%"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="+0.0%;-0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,25 +34,23 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00595959"/>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00B00000"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -63,67 +60,19 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="007F7F7F"/>
+      <color rgb="007A5C00"/>
       <sz val="9"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="009C6500"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="009C0006"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00006100"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E2F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -131,110 +80,36 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -310,6 +185,153 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sessions — semaines calendaires complètes</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Trafic'!B61</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Trafic'!$A$62:$A$66</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Trafic'!$B$62:$B$66</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Semaine</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Sessions</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>60</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -601,13 +623,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -620,790 +642,848 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Semaine du 06/07 au 12/07/2026, comparée à la semaine du 29/06 au 05/07/2026 | Propriété GA4 : ScopIOM (properties/540680472) | Généré le 17/07/2026</t>
+          <t>Semaine du 06/07 au 12/07/2026, comparée à la semaine du 29/06 au 05/07/2026 | Propriété GA4 : ScopIOM (properties/540680472) | Généré le 18/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>⚠ Exécution hors cycle (lancée un samedi, hors du créneau habituel du lundi 8h) : au 18/07/2026, la dernière semaine calendaire complète (lundi-dimanche) reste le 06/07-12/07 — la semaine du 13/07-19/07 ne sera complète que le 19/07. Cette exécution rafraîchit donc le rapport de cette même semaine (déjà produit le 17/07/2026) principalement pour ajouter le graphique d'évolution ci-dessous (nouvelle exigence du 18/07/2026). Toutes les données ont été revérifiées en direct : GA4, Search Console et le crawl Semrush Site Audit sont inchangés depuis le 17/07 ; seuls deux compteurs Semrush (rang de domaine, mots-clés organiques de sealsystems.fr) ont légèrement bougé, voir onglet Concurrence.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Indicateurs clés (volumes)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Indicateur</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Semaine 29/06-05/07</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Semaine 06/07-12/07</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Delta (%)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Sessions</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="6">
         <f>IFERROR((C6-B6)/B6,"n/a")</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Utilisateurs (total)</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="6">
         <f>IFERROR((C7-B7)/B7,"n/a")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Nouveaux utilisateurs</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="6">
         <f>IFERROR((C8-B8)/B8,"n/a")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Pages vues</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="5" t="n">
         <v>525</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="5" t="n">
         <v>692</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="6">
         <f>IFERROR((C9-B9)/B9,"n/a")</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Sessions engagées</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="5" t="n">
         <v>71</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="6">
         <f>IFERROR((C10-B10)/B10,"n/a")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Durée d'engagement cumulée (secondes)</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="5" t="n">
         <v>11527</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="5" t="n">
         <v>17209</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="6">
         <f>IFERROR((C11-B11)/B11,"n/a")</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Indicateurs clés (taux — delta exprimé en points)</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Indicateur</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Semaine 29/06-05/07</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Semaine 06/07-12/07</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Delta (points)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Taux de rebond</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="7" t="n">
         <v>0.4242424242424243</v>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="7" t="n">
         <v>0.1744186046511628</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="6">
         <f>C15-B15</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Taux d'engagement</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="7" t="n">
         <v>0.5757575757575758</v>
       </c>
-      <c r="C16" s="10" t="n">
+      <c r="C16" s="7" t="n">
         <v>0.8255813953488372</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="6">
         <f>C16-B16</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Top 10 pages — semaine du 06/07 au 12/07</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Page (pagePath)</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Pages vues</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Sessions</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>ScopIOM - Logiciel d'Output Management - MPI Tech</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
+      <c r="C20" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="5" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>/ressources-output-management/blog-output-management-editique/</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Blog Output Management &amp; éditique - ScopIOM</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n">
+      <c r="C21" s="5" t="n">
         <v>54</v>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="5" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>ScopIOM – Plateforme d'Output Management et d'orchestration des flux éditiques</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n">
+      <c r="C22" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="5" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>/fonctionnalites-gestion-impressions-editique/ordonnancement-automatisation-des-flux/</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Ordonnancement des flux documentaires - ScopIOM</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C23" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="D23" s="5" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>/fonctionnalites-gestion-impressions-editique/module-workflow/</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Module Workflow : orchestration documentaire no-code - ScopIOM</t>
         </is>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="5" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>/cas-usage-output-management/module-workflow/</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Module Workflow : orchestration documentaire no-code – ScopIOM</t>
         </is>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C25" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="D25" s="7" t="n">
+      <c r="D25" s="5" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>/fonctionnalites-gestion-impressions-editique/</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Fonctionnalités ScopIOM : ordonnancement, distribution et spooling - ScopIOM</t>
         </is>
       </c>
-      <c r="C26" s="7" t="n">
+      <c r="C26" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="D26" s="7" t="n">
+      <c r="D26" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>/ressources-output-management/faq-output-management-questions-frequentes/</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>FAQ output management : déploiement, SAP, HA, sécurité - ScopIOM</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n">
+      <c r="C27" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="D27" s="7" t="n">
+      <c r="D27" s="5" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>/ressources-output-management/blog-output-management-editique/</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Blog Output Management &amp; éditique – ScopIOM</t>
         </is>
       </c>
-      <c r="C28" s="7" t="n">
+      <c r="C28" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="D28" s="7" t="n">
+      <c r="D28" s="5" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>/fonctionnalites-gestion-impressions-editique/module-workflow/</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Module Workflow : orchestration documentaire no-code – ScopIOM</t>
         </is>
       </c>
-      <c r="C29" s="7" t="n">
+      <c r="C29" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="D29" s="7" t="n">
+      <c r="D29" s="5" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>Note : deux lignes '/' et deux lignes 'module-workflow' apparaissent avec des titres légèrement différents (variantes de balise &lt;title&gt; selon la page d'origine WPML/cache) — donnée brute GA4, non retraitée.</t>
-        </is>
-      </c>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="13" t="n"/>
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Note : deux lignes '/' et deux lignes 'module-workflow' apparaissent avec des titres légèrement différents (variantes de balise &lt;title&gt; selon la page d'origine WPML/cache) — donnée brute GA4, non retraitée. Reconfirmé identique lors de la revérification du 18/07/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Répartition géographique — semaine du 06/07 au 12/07</t>
         </is>
       </c>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Sessions</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>% du total</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B34" s="7" t="n">
+      <c r="B34" s="5" t="n">
         <v>53</v>
       </c>
-      <c r="C34" s="10">
+      <c r="C34" s="7">
         <f>B34/C6</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>Pays-Bas (Netherlands)</t>
         </is>
       </c>
-      <c r="B35" s="7" t="n">
+      <c r="B35" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C35" s="7">
         <f>B35/C6</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>(not set)</t>
         </is>
       </c>
-      <c r="B36" s="7" t="n">
+      <c r="B36" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C36" s="10">
+      <c r="C36" s="7">
         <f>B36/C6</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>États-Unis</t>
         </is>
       </c>
-      <c r="B37" s="7" t="n">
+      <c r="B37" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="7">
         <f>B37/C6</f>
         <v/>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="14" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
         <is>
           <t>⚠ Les 29 sessions Pays-Bas sont 100% en canal direct, sans référent identifiable (voir détail source/support ci-dessous) — probable trafic non qualifié (bot, outil de supervision, VPN) plutôt que de vraies visites DSI françaises. À surveiller, pas à additionner sans réserve à l'audience cible.</t>
         </is>
       </c>
-      <c r="B38" s="12" t="n"/>
-      <c r="C38" s="12" t="n"/>
-      <c r="D38" s="13" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Canaux d'acquisition — semaine du 06/07 au 12/07</t>
         </is>
       </c>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Canal</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>Sessions</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>% du total</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>Direct</t>
         </is>
       </c>
-      <c r="B42" s="7" t="n">
+      <c r="B42" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="C42" s="10">
+      <c r="C42" s="7">
         <f>B42/C6</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="9" t="inlineStr">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>Referral</t>
         </is>
       </c>
-      <c r="B43" s="7" t="n">
+      <c r="B43" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="C43" s="10">
+      <c r="C43" s="7">
         <f>B43/C6</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="9" t="inlineStr">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="B44" s="7" t="n">
+      <c r="B44" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C44" s="10">
+      <c r="C44" s="7">
         <f>B44/C6</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="9" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>Organic Search</t>
         </is>
       </c>
-      <c r="B45" s="7" t="n">
+      <c r="B45" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C45" s="10">
+      <c r="C45" s="7">
         <f>B45/C6</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>Détail des sources/supports (semaine courante)</t>
         </is>
       </c>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Pays</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>Source / Support</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Sessions</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="9" t="inlineStr">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>Pays-Bas</t>
         </is>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>(direct) / (none)</t>
         </is>
       </c>
-      <c r="C49" s="7" t="n">
+      <c r="C49" s="5" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="9" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>(direct) / (none)</t>
         </is>
       </c>
-      <c r="C50" s="7" t="n">
+      <c r="C50" s="5" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>brokenlinkcheck.com / referral — outil automatisé de vérification de liens</t>
         </is>
       </c>
-      <c r="C51" s="7" t="n">
+      <c r="C51" s="5" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="inlineStr">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>(not set)</t>
         </is>
       </c>
-      <c r="C52" s="7" t="n">
+      <c r="C52" s="5" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>stg-scopiom-staging.kinsta.cloud / referral — site de staging interne</t>
         </is>
       </c>
-      <c r="C53" s="7" t="n">
+      <c r="C53" s="5" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="9" t="inlineStr">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>(not set)</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>(direct) / (none)</t>
         </is>
       </c>
-      <c r="C54" s="7" t="n">
+      <c r="C54" s="5" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="9" t="inlineStr">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>google / organic</t>
         </is>
       </c>
-      <c r="C55" s="7" t="n">
+      <c r="C55" s="5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="9" t="inlineStr">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>États-Unis</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>(direct) / (none)</t>
         </is>
       </c>
-      <c r="C56" s="7" t="n">
+      <c r="C56" s="5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="9" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>États-Unis</t>
         </is>
       </c>
-      <c r="B57" s="6" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>google / organic</t>
         </is>
       </c>
-      <c r="C57" s="7" t="n">
+      <c r="C57" s="5" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="58" ht="40" customHeight="1">
-      <c r="A58" s="14" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
         <is>
           <t>Constat : brokenlinkcheck.com (16 sessions) est un outil tiers de vérification de liens, pas un visiteur humain. Cumulé aux 29 sessions Pays-Bas non expliquées, jusqu'à 45 sessions sur 86 (≈52%) sont potentiellement non qualifiées cette semaine. La hausse de trafic (+160,6% sessions) doit donc être lue avec prudence — voir onglet Alertes.</t>
         </is>
       </c>
-      <c r="B58" s="12" t="n"/>
-      <c r="C58" s="12" t="n"/>
-      <c r="D58" s="13" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>Évolution des sessions — semaines calendaires complètes (limité à 5 semaines : la propriété GA4 a été créée le 08/06/2026, il n'existe donc pas encore 8 semaines complètes d'historique)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Semaine (lundi-dimanche)</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>08/06-14/06/2026</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>15/06-21/06/2026</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>22/06-28/06/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>29/06-05/07/2026</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>06/07-12/07/2026</t>
+        </is>
+      </c>
+      <c r="B66" s="5">
+        <f>C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>Note : la somme jour par jour de cette dernière semaine (GA4, dimension 'date') donne 87 sessions contre 86 pour l'agrégat par propriété utilisé partout ailleurs dans ce rapport — écart de 1 typique du seuillage de confidentialité GA4 sur une propriété à faible volume ('data thresholding'). La valeur 86 (liée par formule à C6) est retenue pour rester cohérente avec le reste du rapport.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
+    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A38:D38"/>
     <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A60:D60"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1413,12 +1493,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1433,108 +1513,105 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Propriété : https://scopiom.com/ | Semaine du 06/07 au 12/07/2026 vs 29/06 au 05/07/2026</t>
+          <t>Propriété : https://scopiom.com/ | Semaine du 06/07 au 12/07/2026 vs 29/06 au 05/07/2026 | Revérifié le 18/07/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Indicateurs globaux (agrégation par propriété)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Indicateur</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Semaine 29/06-05/07</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Semaine 06/07-12/07</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Delta</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Clics</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="5">
         <f>IF(B6=0,"n/a (base à 0)",(C6-B6)/B6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="5">
         <f>IF(B7=0,"n/a (base à 0)",(C7-B7)/B7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>CTR</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="7" t="n">
         <v>0.1428571428571428</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="6">
         <f>C8-B8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Position moyenne</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>n/a (0 impression)</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="5" t="n">
         <v>4.214285714285714</v>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>n/a (pas de base de comparaison)</t>
         </is>
@@ -1546,213 +1623,203 @@
           <t>Position moyenne = moyenne pondérée par les impressions (donnée Search Console). CTR delta exprimé en points.</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Requêtes visibles — semaine du 06/07 au 12/07</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Requête</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Clics</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>CTR</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>scopiom</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E14" s="5" t="n">
         <v>3.7</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>plateforme / solution / logiciel output management</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="16" t="n">
+      <c r="E15" s="5" t="n">
         <v>19</v>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Search Console masque les requêtes individuelles à très faible volume pour des raisons de confidentialité : la somme des lignes ci-dessus (1 clic / 11 impressions) est donc inférieure au total agrégé de la semaine (2 clics / 14 impressions ci-dessus) — écart normal, pas une anomalie.</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Nouvelles requêtes apparues cette semaine</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Requête</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>scopiom</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n">
+      <c r="B20" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Nouvelle (0 impression la semaine précédente)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>plateforme / solution / logiciel output management</t>
         </is>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B21" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Nouvelle (0 impression la semaine précédente)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Pages — progression semaine sur semaine</t>
         </is>
       </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Page</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Clics/Impr. semaine préc.</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Clics/Impr. semaine courante</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Évolution</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>https://scopiom.com/</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>0 / 0</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>2 / 14</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Nouvelle visibilité — seule page avec impressions sur les deux semaines analysées</t>
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Revérification du 18/07/2026 : données Search Console identiques à celles du rapport du 17/07/2026, aucun changement.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A27:E27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1764,14 +1831,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1784,323 +1851,300 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Base régionale : France (fr) | Données actualisées le 17/07/2026</t>
+          <t>Base régionale : France (fr) | Données actualisées le 18/07/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Comparatif de domaines — Semrush Domain Overview</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Domaine</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Semrush Rank</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Mots-clés organiques</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Trafic organique estimé/mois</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Coût trafic estimé</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>scopiom.com</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>0 $</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>sealsystems.fr</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
-        <v>343928</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>576</v>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="B7" s="5" t="n">
+        <v>345117</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>201</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>574</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>368 $</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>scopiom.com n'a aucun mot-clé indexé dans la base Semrush FR (inchangé depuis le rapport précédent). Les chiffres SEAL Systems sont identiques à l'instantané précédent — Semrush ne semble pas avoir rafraîchi ce domaine cette semaine ; ces totaux ne reflètent donc pas nécessairement une évolution réelle de la semaine.</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="13" t="n"/>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>scopiom.com n'a toujours aucun mot-clé indexé dans la base Semrush FR (inchangé). Pour sealsystems.fr, très légère variation vs le rapport du 17/07/2026 : rang 345117 (vs 343928), 201 mots-clés organiques (vs 200), trafic estimé 574/mois (vs 576) — fluctuations mineures de rafraîchissement Semrush, pas une évolution significative de sa visibilité.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>SERP en direct — mot-clé prioritaire "output management system" (base FR, requête du 17/07/2026)</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>SERP en direct — mot-clé prioritaire "output management system" (base FR, requête du 18/07/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Domaine</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="n">
+      <c r="A12" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>sefasinnovation.fr</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>/output-management</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>sealsystems.fr</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>/blog/output-management-pourquoi-les-entreprises-doivent-s-y-interesser/</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="n">
+      <c r="A14" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>betasystems.com</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>/resources/blog/what-is-output-management</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="n">
+      <c r="A15" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>nazdaq-it.com</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>/resources/blog/what-is-an-output-management-system-oms</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="n">
+      <c r="A16" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>vasion.com</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>/fr/blog/redefining-output-management/</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="n">
+      <c r="A17" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>mpitech.com  ⚠ (MPI Tech, pas scopiom.com)</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>/output-management-systems-guide/</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>scopiom.com</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Absent du top 20</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="55" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>⚠ CHANGEMENT DE RAPPORT DE FORCE : Sefas Innovation (sefasinnovation.fr) occupe désormais la position 1 sur "output management system" (base FR) — SEAL Systems recule en position 2. CLAUDE.md §3/§4.4 désignait encore SEAL Systems comme le concurrent en position 1 à battre sur la base du snapshot Semrush d'avril 2026 ; cette donnée est obsolète (mise à jour appliquée dans CLAUDE.md ce jour, voir commit du rapport).</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="13" t="n"/>
-    </row>
-    <row r="20" ht="55" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>⚠ MPI Tech (l'éditeur de ScopIOM) se positionne déjà en position 7 avec une page sur mpitech.com, alors que scopiom.com — le site produit dédié, pivot de toute la stratégie SEO du §3 — n'apparaît nulle part dans le top 20 pour ce mot-clé prioritaire n°1. Risque de dispersion d'autorité / cannibalisation entre les deux domaines à examiner avec l'équipe web (faut-il rediriger/consolider ce contenu vers scopiom.com ?).</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="13" t="n"/>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Situation inchangée depuis le rapport du 17/07/2026 : Sefas Innovation reste en position 1, SEAL Systems en position 2, MPI Tech (mpitech.com, pas scopiom.com) en position 7. Aucun mouvement de position cette semaine sur ce mot-clé prioritaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Veille concurrentielle — blog SEAL Systems (CLAUDE.md §7)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Veille concurrentielle — blog SEAL Systems (CLAUDE.md §7)</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Dernière vérification :</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>17/07/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>18/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Résultat :</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Aucun nouvel article depuis la dernière entrée connue (13/07/2026 — "Impressions SAP : le REX d'un groupe de luxe dans l'USF Mag n°70"). Liste inchangée par rapport à CLAUDE.md. Rythme de publication d'environ 2 semaines confirmé (dernier article il y a 4 jours, prochain probablement fin juillet).</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="13" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Aucun nouvel article depuis le 13/07/2026 ("Impressions SAP : le REX d'un groupe de luxe dans l'USF Mag n°70"), reconfirmé par une nouvelle vérification directe de la page blog. Liste inchangée par rapport à CLAUDE.md et au rapport du 17/07/2026. Rythme de publication d'environ 2 semaines confirmé (dernier article il y a 5 jours, prochain probablement fin juillet/début août).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Statut campagne Position Tracking Semrush (CLAUDE.md §5.4)</t>
         </is>
       </c>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-    </row>
-    <row r="27" ht="65" customHeight="1">
-      <c r="A27" s="20" t="inlineStr">
-        <is>
-          <t>Les deux projets Semrush existants ("ScopIOM - SEO", id 30407302, et "ScopIOM - IA", id 30404738) ont l'outil de tracking activé mais AUCUNE campagne de suivi de position n'y est configurée à ce jour (0 mot-clé cible). La campagne à 34 mots-clés / 6 clusters décrite en §5.4 n'existe donc pas dans Semrush : impossible d'obtenir des mouvements de position semaine/semaine ni d'alerter sur une sortie du top 10 tant qu'elle n'est pas créée. Action recommandée : créer la campagne de Position Tracking dans le projet "ScopIOM - SEO".</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="n"/>
-      <c r="C27" s="12" t="n"/>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="13" t="n"/>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Reconfirmé le 18/07/2026 : les deux projets Semrush existants ("ScopIOM - SEO", id 30407302, et "ScopIOM - IA", id 30404738) ont l'outil de tracking activé mais AUCUNE campagne de suivi de position n'y est configurée (0 mot-clé cible). Impossible d'obtenir des mouvements de position semaine/semaine ni d'alerter sur une sortie du top 10 tant qu'elle n'est pas créée. Action recommandée : créer la campagne de Position Tracking dans le projet "ScopIOM - SEO".</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Technique (Semrush Site Audit — CLAUDE.md §2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>Dernier crawl disponible : 13/07/2026 (36 pages), aucun nouveau crawl cette semaine — projet "ScopIOM - SEO", 0 page "broken" (4xx/5xx), 0 page bloquée, errors_delta = 0 (2 erreurs persistantes = conflit schema FAQPage/Rank Math déjà connu, cf. CLAUDE.md §2). Ce chiffre n'a donc pas pu être rafraîchi cette semaine ; il reste la donnée la plus récente disponible.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A20:E20"/>
+  <mergeCells count="6">
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A19:E19"/>
-    <mergeCell ref="B24:E24"/>
     <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A27:E27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2112,12 +2156,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2135,137 +2179,154 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Type d'alerte</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Détail</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="55" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Chute de trafic &gt; 15% vs semaine précédente</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Aucune</t>
         </is>
       </c>
-      <c r="C5" s="6">
-        <f>"Sessions "&amp;TEXT(Trafic!D6,"+0.0%;-0.0%")&amp;", utilisateurs "&amp;TEXT(Trafic!D7,"+0.0%;-0.0%")&amp;" vs semaine précédente — hausse sur tous les indicateurs, pas de chute. Voir réserve sur la qualité du trafic ci-dessous."</f>
+      <c r="C5" s="13">
+        <f>"Sessions "&amp;TEXT(Trafic!D6,"+0.0%;-0.0%")&amp;", utilisateurs "&amp;TEXT(Trafic!D7,"+0.0%;-0.0%")&amp;" vs semaine précédente — hausse sur tous les indicateurs, pas de chute. Voir réserve sur la qualité du trafic ci-dessous.</f>
         <v/>
       </c>
     </row>
-    <row r="6" ht="55" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Nouvelle page en erreur 404/500</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Aucune détectée</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Semrush Site Audit (crawl du 13/07/2026, projet "ScopIOM - SEO", 36 pages explorées) : 0 page "broken" (4xx/5xx), 0 page bloquée. 2 erreurs de structured data persistent (conflit schema FAQPage/Rank Math déjà connu, cf. CLAUDE.md §2, dette technique) — ce n'est pas une régression de la semaine (errors_delta = 0).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="55" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Semrush Site Audit : dernier crawl disponible du 13/07/2026 (projet "ScopIOM - SEO", 36 pages), reconfirmé identique le 18/07/2026 — 0 page "broken" (4xx/5xx), 0 page bloquée, errors_delta = 0. Aucun nouveau crawl ne s'est déclenché cette semaine ; ce n'est donc pas une confirmation fraîche mais la persistance du dernier état connu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Mot-clé prioritaire sorti du top 10</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Non applicable</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>scopiom.com n'a aujourd'hui aucun mot-clé positionné dans le top 100 Semrush (base FR, 0 mot-clé organique indexé) : rien ne peut donc "sortir" du top 10 cette semaine, la situation de départ est déjà hors classement. Cette alerte redeviendra pertinente une fois les premiers mots-clés indexés.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="55" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Qualité du trafic (hors seuils standards du cahier des charges)</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>À surveiller</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Sur 86 sessions cette semaine, 29 (Pays-Bas, 100% direct/sans référent) et 16 (France, référent brokenlinkcheck.com — outil automatisé de vérification de liens) semblent non qualifiées, soit environ 52% du volume. La hausse de trafic affichée dans l'onglet Trafic (+160,6% sessions) doit être lue avec cette réserve — recommandé : exclure ces sources dans GA4 (filtre trafic interne/bot) avant le prochain rapport.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="55" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Campagne Position Tracking Semrush vide</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>À corriger</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Voir onglet Concurrence : les projets Semrush existants n'ont aucune campagne de suivi de mots-clés configurée. Aucune donnée de mouvement de position disponible tant que la campagne n'est pas créée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="55" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Voir onglet Concurrence : les projets Semrush existants n'ont toujours aucune campagne de suivi de mots-clés configurée (reconfirmé le 18/07/2026). Aucune donnée de mouvement de position disponible tant que la campagne n'est pas créée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Changement de position SERP "output management system"</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Aucun changement cette semaine</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Sefas Innovation reste en position 1, SEAL Systems en position 2 (base FR) — situation identique à celle déjà signalée dans le rapport du 17/07/2026, pas un nouveau mouvement cette semaine. MPI Tech (mpitech.com, pas scopiom.com) reste en position 7. Voir onglet Concurrence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Veille SEAL Systems (blog)</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Aucun nouvel article</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Revérifié le 18/07/2026 : aucun article publié depuis le 13/07/2026 (dernier connu). Voir onglet Concurrence pour le détail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Exécution hors cycle (nouveau, cette exécution)</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Information</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>SEAL Systems recule de la position 1 à la position 2 sur ce mot-clé prioritaire (base FR) ; Sefas Innovation (sefasinnovation.fr) prend la tête. MPI Tech (mpitech.com, pas scopiom.com) est en position 7. Voir onglet Concurrence pour le détail et l'impact sur la stratégie éditoriale du §3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="55" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>Veille SEAL Systems (blog)</t>
-        </is>
-      </c>
-      <c r="B11" s="22" t="inlineStr">
-        <is>
-          <t>Aucun nouvel article</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Vérifié le 17/07/2026 : aucun article publié depuis le 13/07/2026 (dernier connu). Voir onglet Concurrence pour le détail.</t>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Cette exécution s'est déclenchée le 18/07/2026 (samedi), hors du créneau habituel du lundi 8h. Aucune nouvelle semaine calendaire complète n'a pu s'écouler depuis le dernier rapport (17/07/2026) : ce rapport porte donc sur la même semaine (06/07-12/07) et sert principalement à ajouter le graphique d'évolution des sessions sur l'onglet Trafic, nouvelle exigence du 18/07/2026. Le prochain rapport hebdomadaire réellement nouveau est attendu lundi 20/07/2026 pour la semaine 13/07-19/07.</t>
         </is>
       </c>
     </row>

</xml_diff>